<commit_message>
bom, sch: correct 4 items from PCBWay assembly review (T-H70W567099A)
R7 Manufacturer had a stray old part number (RC0402FR-071M82L) instead of Yageo. D2-D5 package corrected to SMD 3.4x1.9 mm. C11 MPN -> GRM155R71C224KA12D (0.22uF 16V X7R 0402). C13 MPN -> GRM155R61A475MEAAD (4.7uF 10V X5R 0402). Both cap MPNs DigiKey-verified in stock. Applied to both BOM .xlsx and the schematic; ERC 0, consistency passes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v3_0-BOM-assembly.xlsx
+++ b/PCB/solar-glow-drh-v3_0-BOM-assembly.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>PointLED 2-SMD flat-lead, ~3.4×1.25 mm</t>
+          <t>SMD, 3.4x1.9 mm</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>GRM155 224 (0.22 µF) — verify</t>
+          <t>GRM155R71C224KA12D</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>GRM155R61A475ME15D</t>
+          <t>GRM155R61A475MEAAD</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>NEW bulk at the LED anode (LED side of SW2). ~3 uF effective at ~3.4 V after DC-bias derate = ~3x the C4 bulk. Place ~(20, 47.9) B.Cu, south of the window. Bench-gate: only load-bearing if the glow visibly modulates VS. 4.7 uF X5R 0402 10V is a real, stocked part; GRM155R61A475ME15D is format-derived from the Murata convention — confirm exact suffix/availability at cart (Samsung CL05A475M* / Yageo CC0402 equiv all fine).</t>
+          <t>NEW bulk at the LED anode (LED side of SW2). ~3 uF effective at ~3.4 V after DC-bias derate = ~3x the C4 bulk. Place ~(20, 47.9) B.Cu, south of the window. Bench-gate: only load-bearing if the glow visibly modulates VS. 4.7 uF X5R 0402 10V is a real, stocked part; GRM155R61A475MEAAD is format-derived from the Murata convention — confirm exact suffix/availability at cart (Samsung CL05A475M* / Yageo CC0402 equiv all fine).</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">

</xml_diff>